<commit_message>
Created excel sheet for soil data
</commit_message>
<xml_diff>
--- a/Lab-trails/2026-01-06-cattle-slurry/Lab 1 overview.xlsx
+++ b/Lab-trails/2026-01-06-cattle-slurry/Lab 1 overview.xlsx
@@ -5,22 +5,21 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mikae\Desktop\Github - speciale\Larsen-2025-Masterthesis-DFCs\Lab-acidification-field-and-lab-comparision\Lab plans\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mikae\Desktop\Github - speciale\Larsen-2025-Masterthesis-DFCs\Lab-trails\2026-01-06-cattle-slurry\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD0C3D76-1EED-490E-9A63-EFDF54815999}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D386DE2-889B-4DEF-817A-F1E024F35FD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-2820" windowWidth="38640" windowHeight="21120" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Jar and valve ids" sheetId="1" r:id="rId1"/>
-    <sheet name="Picarro plan1" sheetId="8" r:id="rId2"/>
-    <sheet name="Picarro plan 2 " sheetId="9" r:id="rId3"/>
-    <sheet name="Slurry pH" sheetId="2" r:id="rId4"/>
-    <sheet name="soil pH" sheetId="3" r:id="rId5"/>
-    <sheet name="TAN" sheetId="4" r:id="rId6"/>
-    <sheet name="DM" sheetId="5" r:id="rId7"/>
-    <sheet name="Field-soil water content" sheetId="6" r:id="rId8"/>
+    <sheet name="Picarro plan 2 " sheetId="9" r:id="rId2"/>
+    <sheet name="Slurry pH" sheetId="2" r:id="rId3"/>
+    <sheet name="soil pH" sheetId="3" r:id="rId4"/>
+    <sheet name="TAN" sheetId="4" r:id="rId5"/>
+    <sheet name="DM" sheetId="5" r:id="rId6"/>
+    <sheet name="Field-soil water content" sheetId="6" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -45,24 +44,6 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
-    <author>tc={EAE3A72D-FDAA-4985-8621-C558E5893AC1}</author>
-  </authors>
-  <commentList>
-    <comment ref="C25" authorId="0" shapeId="0" xr:uid="{EAE3A72D-FDAA-4985-8621-C558E5893AC1}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    10 s</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
     <author>Mikael Løvig Larsen</author>
   </authors>
   <commentList>
@@ -74,7 +55,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Mikael Løvig Larsen:</t>
         </r>
@@ -83,7 +64,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 no container mass</t>
@@ -95,7 +76,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="47">
   <si>
     <t>Picarro ID</t>
   </si>
@@ -172,18 +153,9 @@
     <t>Background</t>
   </si>
   <si>
-    <t>Control</t>
-  </si>
-  <si>
     <t>P H2SO4</t>
   </si>
   <si>
-    <t>F Untreated</t>
-  </si>
-  <si>
-    <t>P Untreated</t>
-  </si>
-  <si>
     <t>F H2SO4</t>
   </si>
   <si>
@@ -191,12 +163,6 @@
   </si>
   <si>
     <t>P AA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F AA </t>
-  </si>
-  <si>
-    <t>P untreated</t>
   </si>
   <si>
     <t>Field a</t>
@@ -260,7 +226,7 @@
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
-    <numFmt numFmtId="168" formatCode="#,##0.0000"/>
+    <numFmt numFmtId="166" formatCode="#,##0.0000"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -274,14 +240,14 @@
       <sz val="9"/>
       <color indexed="81"/>
       <name val="Tahoma"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="9"/>
       <color indexed="81"/>
       <name val="Tahoma"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -323,7 +289,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -342,9 +308,7 @@
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <person displayName="Mikael Løvig Larsen" id="{703632F6-CAB6-4F7B-B593-D79EDDAB58DB}" userId="S::au705323@uni.au.dk::501b5c6e-34b9-41fc-bcf2-dc0650cde639" providerId="AD"/>
-</personList>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -608,14 +572,6 @@
 </a:theme>
 </file>
 
-<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
-<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="C25" dT="2026-01-05T14:55:14.23" personId="{703632F6-CAB6-4F7B-B593-D79EDDAB58DB}" id="{EAE3A72D-FDAA-4985-8621-C558E5893AC1}">
-    <text>10 s</text>
-  </threadedComment>
-</ThreadedComments>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C25"/>
@@ -850,323 +806,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{784E99AC-3353-4400-B6CB-8B44B2AAC519}">
-  <dimension ref="A1:K25"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="3" max="3" width="15.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="20.77734375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.21875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.44140625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="C2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3">
-        <v>2</v>
-      </c>
-      <c r="C3" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4">
-        <v>3</v>
-      </c>
-      <c r="C4" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5">
-        <v>4</v>
-      </c>
-      <c r="C5" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6">
-        <v>5</v>
-      </c>
-      <c r="C6" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7">
-        <v>6</v>
-      </c>
-      <c r="C7" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8">
-        <v>7</v>
-      </c>
-      <c r="C8" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A9" s="1">
-        <v>11</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A10">
-        <v>8</v>
-      </c>
-      <c r="B10">
-        <v>8</v>
-      </c>
-      <c r="C10" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A11">
-        <v>9</v>
-      </c>
-      <c r="B11">
-        <v>9</v>
-      </c>
-      <c r="C11" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A12">
-        <v>10</v>
-      </c>
-      <c r="B12">
-        <v>10</v>
-      </c>
-      <c r="C12" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A13">
-        <v>17</v>
-      </c>
-      <c r="B13">
-        <v>11</v>
-      </c>
-      <c r="C13" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A14">
-        <v>18</v>
-      </c>
-      <c r="B14">
-        <v>12</v>
-      </c>
-      <c r="C14" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A15">
-        <v>19</v>
-      </c>
-      <c r="B15">
-        <v>13</v>
-      </c>
-      <c r="C15" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A16">
-        <v>20</v>
-      </c>
-      <c r="B16">
-        <v>14</v>
-      </c>
-      <c r="C16" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="1">
-        <v>12</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18">
-        <v>21</v>
-      </c>
-      <c r="B18">
-        <v>15</v>
-      </c>
-      <c r="C18" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19">
-        <v>22</v>
-      </c>
-      <c r="B19">
-        <v>16</v>
-      </c>
-      <c r="C19" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20">
-        <v>23</v>
-      </c>
-      <c r="B20">
-        <v>17</v>
-      </c>
-      <c r="C20" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21">
-        <v>24</v>
-      </c>
-      <c r="B21">
-        <v>18</v>
-      </c>
-      <c r="C21" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22">
-        <v>25</v>
-      </c>
-      <c r="B22">
-        <v>19</v>
-      </c>
-      <c r="C22" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23">
-        <v>26</v>
-      </c>
-      <c r="B23">
-        <v>20</v>
-      </c>
-      <c r="C23" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" s="1">
-        <v>27</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25">
-        <v>28</v>
-      </c>
-      <c r="B25" t="s">
-        <v>2</v>
-      </c>
-      <c r="C25" t="s">
-        <v>24</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A713999E-2F40-4260-ADE4-77E01BA78E57}">
-  <dimension ref="A1:L33"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.88671875" bestFit="1" customWidth="1"/>
@@ -1181,10 +822,10 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="B1" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -1225,7 +866,7 @@
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="E2">
         <v>2.04</v>
@@ -1245,7 +886,7 @@
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="E3">
         <v>2.1349999999999998</v>
@@ -1262,7 +903,7 @@
         <v>3</v>
       </c>
       <c r="D4" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="E4">
         <v>2.0219999999999998</v>
@@ -1279,7 +920,7 @@
         <v>4</v>
       </c>
       <c r="D5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E5">
         <v>2.0499999999999998</v>
@@ -1296,7 +937,7 @@
         <v>5</v>
       </c>
       <c r="D6" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="E6">
         <v>2.097</v>
@@ -1327,7 +968,7 @@
         <v>6</v>
       </c>
       <c r="D8" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E8">
         <v>2.0710000000000002</v>
@@ -1344,7 +985,7 @@
         <v>7</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="E9">
         <v>2.0819999999999999</v>
@@ -1361,7 +1002,7 @@
         <v>8</v>
       </c>
       <c r="D10" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="E10" s="2">
         <v>2.02</v>
@@ -1378,7 +1019,7 @@
         <v>9</v>
       </c>
       <c r="D11" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="E11" s="2">
         <v>2.08</v>
@@ -1395,7 +1036,7 @@
         <v>10</v>
       </c>
       <c r="D12" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E12" s="2">
         <v>2.0299999999999998</v>
@@ -1426,7 +1067,7 @@
         <v>11</v>
       </c>
       <c r="D14" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="E14" s="2">
         <v>2.0299999999999998</v>
@@ -1443,7 +1084,7 @@
         <v>12</v>
       </c>
       <c r="D15" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="E15" s="2">
         <v>2.1070000000000002</v>
@@ -1460,7 +1101,7 @@
         <v>13</v>
       </c>
       <c r="D16" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="E16" s="2">
         <v>2.0419999999999998</v>
@@ -1477,7 +1118,7 @@
         <v>14</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="E17" s="2">
         <v>2.02</v>
@@ -1494,7 +1135,7 @@
         <v>15</v>
       </c>
       <c r="D18" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E18" s="2">
         <v>2.0649999999999999</v>
@@ -1525,7 +1166,7 @@
         <v>16</v>
       </c>
       <c r="D20" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E20" s="2">
         <v>2.0870000000000002</v>
@@ -1542,7 +1183,7 @@
         <v>17</v>
       </c>
       <c r="D21" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="E21" s="2">
         <v>2.0390000000000001</v>
@@ -1559,7 +1200,7 @@
         <v>18</v>
       </c>
       <c r="D22" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="E22" s="2">
         <v>2.09</v>
@@ -1576,7 +1217,7 @@
         <v>19</v>
       </c>
       <c r="D23" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E23" s="2">
         <v>2.0979999999999999</v>
@@ -1593,7 +1234,7 @@
         <v>20</v>
       </c>
       <c r="D24" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="E24" s="2">
         <v>2.0859999999999999</v>
@@ -1611,36 +1252,6 @@
       </c>
       <c r="D25" s="1" t="s">
         <v>24</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A30" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A32" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
-        <v>44</v>
       </c>
     </row>
   </sheetData>
@@ -1648,7 +1259,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C34E2B22-EFBB-47A1-AF0B-5767E9B20688}">
   <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1736,7 +1347,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDD98347-804C-4072-BF54-67982692E8A8}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1751,7 +1362,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F78E8D4-D646-46E6-89EC-8C44B7945A50}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1766,29 +1377,29 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C2A4B67-C43D-42B5-8319-7D9C81B9E3D4}">
   <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="B1" t="s">
         <v>3</v>
       </c>
       <c r="C1" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="D1" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
@@ -1796,7 +1407,7 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="C2" s="5">
         <v>30.201000000000001</v>
@@ -1810,7 +1421,7 @@
         <v>9</v>
       </c>
       <c r="B3" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="C3">
         <v>31.4588</v>
@@ -1824,7 +1435,7 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="C4">
         <v>31.767600000000002</v>
@@ -1923,13 +1534,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65F4B115-3694-4A6B-99C0-95DC5F83777D}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="10.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
@@ -1943,12 +1554,12 @@
         <v>22</v>
       </c>
       <c r="D1" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="B2">
         <v>4.26</v>
@@ -1962,7 +1573,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="B3">
         <v>4.2619999999999996</v>
@@ -1976,7 +1587,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="B4" s="2">
         <v>4.28</v>
@@ -1990,7 +1601,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B5" s="2">
         <v>4.2699999999999996</v>
@@ -2004,7 +1615,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B6">
         <v>4.2729999999999997</v>
@@ -2018,7 +1629,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B7">
         <v>4.2729999999999997</v>

</xml_diff>